<commit_message>
365 by Whole Foods: regrade with the unknown rule (no Puberty Safe with unknown ingredients); dashboard updated
Co-Authored-By: Claude Haiku 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QozUH5QDLofYCKpqXvk3Fh
</commit_message>
<xml_diff>
--- a/audits/wf365/wf365_audit.xlsx
+++ b/audits/wf365/wf365_audit.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="365 by Whole Foods Audit" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="audit" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -524,22 +524,26 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Cocamidopropyl Hydroxysultaine [1,4] / Parfum [1,2,4,8] / Guar Hydroxypropyltrimonium Chloride [2]</t>
+          <t>Cocamidopropyl Hydroxysultaine [1,4] / Parfum [1,2,4,8] (fragrance without disclosure) / Guar Hydroxypropyltrimonium Chloride [2]</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Sodium Methyl 2-Sulfolaurate, Cetyl Betaine, Disodium 2-Sulfolaurate, Hydrolyzed Rice Protein, Hydrolyzed Collagen</t>
+          <t>unknown — manual review needed: Sodium Methyl 2-Sulfolaurate, Cetyl Betaine, Disodium 2-Sulfolaurate, Tetrasodium Glutamate Diacetate, Hydrolyzed Rice Protein, Hydrolyzed Collagen</t>
         </is>
       </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3 flagged ingredient(s) incl. Cocamidopropyl Hydroxysultaine, Parfum, Guar Hydroxypropyltrimonium Chloride.</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
+          <t>3 flagged ingredient(s) in the printed list (Cocamidopropyl Hydroxysultaine, Parfum, Guar Hydroxypropyltrimonium Chloride); tier applies to the printed subset only. 6 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 6 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>complete</t>
@@ -578,26 +582,30 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Cocamidopropyl Hydroxysultaine [1,4]</t>
+          <t>Cocamidopropyl Hydroxysultaine [1,4] / Polyquaternium-10 [2] (inferred: -nium quat)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Sodium Methyl 2-Sulfolaurate, Disodium 2-Sulfolaurate</t>
+          <t>unknown — manual review needed: Sodium Methyl 2-Sulfolaurate, Disodium 2-Sulfolaurate, Tetrasodium Glutamate Diacetate, Aloe Barbadensis Leaf Extract</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1 flagged ingredient(s) incl. Cocamidopropyl Hydroxysultaine.</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
+          <t>2 flagged ingredient(s) in the printed list (Cocamidopropyl Hydroxysultaine, Polyquaternium-10); tier applies to the printed subset only. 4 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 4 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
           <t>complete</t>
@@ -636,26 +644,30 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Cocamidopropyl Hydroxysultaine [1,4] / Guar Hydroxypropyltrimonium Chloride [2] / Parfum [1,2,4,8]</t>
+          <t>Cocamidopropyl Hydroxysultaine [1,4] / Guar Hydroxypropyltrimonium Chloride [2] / Parfum [1,2,4,8] (fragrance without disclosure) / Polysorbate 20 [1,2,4,5]</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Sodium Methyl 2-Sulfolaurate, Cetyl Betaine, Disodium 2-Sulfolaurate, Hydrolyzed Jojoba Esters</t>
+          <t>unknown — manual review needed: Sodium Methyl 2-Sulfolaurate, Cetyl Betaine, Disodium 2-Sulfolaurate, Hydrolyzed Jojoba Esters, Tetrasodium Glutamate Diacetate, Cannabis Sativa Seed Oil, Argania Spinosa Kernel Oil</t>
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
-          <t>3 flagged ingredient(s) incl. Cocamidopropyl Hydroxysultaine, Guar Hydroxypropyltrimonium Chloride, Parfum.</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr"/>
+          <t>4 flagged ingredient(s) in the printed list (Cocamidopropyl Hydroxysultaine, Guar Hydroxypropyltrimonium Chloride, Parfum); tier applies to the printed subset only. 7 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 7 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
           <t>complete</t>
@@ -694,26 +706,30 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Cetrimonium Chloride [2] / Parfum [1,2,4,8]</t>
+          <t>Cetrimonium Chloride [2] / Parfum [1,2,4,8] (fragrance without disclosure) / Polysorbate 20 [1,2,4,5]</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>C13-15 Alkane, Stearamidopropyl Dimethylamine, Hydrolyzed Jojoba Esters</t>
+          <t>unknown — manual review needed: C13-15 Alkane, Lactic Acid, Stearamidopropyl Dimethylamine, Helianthus Annuus Seed Oil, Hydrolyzed Jojoba Esters, Sodium Hydroxide, Tetrasodium Glutamate Diacetate, Cannabis Sativa Seed Oil, Argania Spinosa Kernel Oil</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2 flagged ingredient(s) incl. Cetrimonium Chloride, Parfum.</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr"/>
+          <t>3 flagged ingredient(s) in the printed list (Cetrimonium Chloride, Parfum, Polysorbate 20); tier applies to the printed subset only. 9 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 9 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
           <t>complete</t>
@@ -760,14 +776,22 @@
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>unknown — manual review needed: Glyceryl Stearate, Cocos Nucifera Oil, Tetrasodium Glutamate Diacetate</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2 flagged ingredient(s) incl. Behentrimonium Chloride, Guar Hydroxypropyltrimonium Chloride.</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr"/>
+          <t>2 flagged ingredient(s) in the printed list (Behentrimonium Chloride, Guar Hydroxypropyltrimonium Chloride); tier applies to the printed subset only. 3 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 3 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
           <t>complete</t>
@@ -806,26 +830,30 @@
         </is>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Cocamidopropyl Betaine [1,4] / Sodium Coco-Sulfate [4,5] / Ammonium Lauryl Sulfate [inferred: sulfate] [1,4,5] / Parfum [1,2,4,8] / Guar Hydroxypropyltrimonium Chloride [2]</t>
+          <t>Cocamidopropyl Betaine [1,4] / Sodium Coco-Sulfate [4,5] / Ammonium Lauryl Sulfate [1,4,5] (inferred: sulfate) / Parfum [1,2,4,8] (fragrance without disclosure) / Polyquaternium-7 [2] (inferred: -nium quat) / Guar Hydroxypropyltrimonium Chloride [2]</t>
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Glycol Stearate, Coconut Alkanes, Coco-Caprylate/Caprate, Hydrolyzed Quinoa</t>
+          <t>unknown — manual review needed: Glycol Stearate, Aloe Barbadensis Leaf Juice, Coco-Betaine, Gluconolactone, Cocos Nucifera Oil, Xylitol, Coco-Caprylate/Caprate, Hydrolyzed Quinoa, Prunus Amygdalus Dulcis Oil, Simmondsia Chinensis Seed Oil</t>
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>5 flagged ingredient(s) incl. Cocamidopropyl Betaine, Sodium Coco-Sulfate, Ammonium Lauryl Sulfate.</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr"/>
+          <t>6 flagged ingredient(s) in the printed list (Cocamidopropyl Betaine, Sodium Coco-Sulfate, Ammonium Lauryl Sulfate); tier applies to the printed subset only. 10 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Sulfate-flagged ingredient in a daily rinse-off product: minimum Avoid (Mild) (rubric, shampoos). D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 10 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
           <t>complete</t>
@@ -864,17 +892,17 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Acrylates Copolymer [1,2,4,6] / Phenoxyethanol [1,2,4,5,8] / Guar Hydroxypropyltrimonium Chloride [2] / Ethylhexylglycerin [4,5] / Hexylene Glycol [1,2]</t>
+          <t>Sodium Cocoyl Isethionate [1] / Acrylates Copolymer [1,2,4,6] / Phenoxyethanol [1,2,4,5,8] / Guar Hydroxypropyltrimonium Chloride [2] / Ethylhexylglycerin [4,5] / Hexylene Glycol [1,2]</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Sodium Laurylglucosides Hydroxypropylsulfonate</t>
+          <t>unknown — manual review needed: Arginine, Sodium Laurylglucosides Hydroxypropylsulfonate, Butyrospermum Parkii Butter, Colloidal Oatmeal</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -884,10 +912,14 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>5 flagged ingredient(s) incl. Acrylates Copolymer, Phenoxyethanol, Guar Hydroxypropyltrimonium Chloride. Escalation: PFAS.</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr"/>
+          <t>6 flagged ingredient(s) in the printed list (Sodium Cocoyl Isethionate, Acrylates Copolymer, Phenoxyethanol); tier applies to the printed subset only. 4 unknown ingredient(s) not in reference, excluded from grade. Escalation: PFAS.</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 4 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
           <t>complete</t>
@@ -922,30 +954,34 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Use Caution</t>
+          <t>Avoid (Mild)</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Phenoxyethanol [1,2,4,5,8]</t>
+          <t>Propanediol [4] / Phenoxyethanol [1,2,4,5,8]</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Sorbitan Caprylate, Sodium Stearoyl Glutamate</t>
+          <t>unknown — manual review needed: Sorbitan Caprylate, Sodium Stearoyl Glutamate, Acrylates/C10-30 Alkyl Acrylate Crosspolymer, Sodium Hydroxide</t>
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1 flagged ingredient(s) incl. Phenoxyethanol.</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr"/>
+          <t>2 flagged ingredient(s) in the printed list (Propanediol, Phenoxyethanol); tier applies to the printed subset only. 4 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>4 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
           <t>complete</t>
@@ -980,7 +1016,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Avoid (High Priority Swap)</t>
+          <t>Use Caution</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -988,22 +1024,26 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Titanium Dioxide [1,2,3]</t>
+          <t>Sodium Cocoyl Isethionate [1]</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>PFAS, heavy metals</t>
-        </is>
-      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>unknown — manual review needed: Butyrospermum Parkii Butter, Theobroma Cacao Seed Butter, Stearic Acid, Tetrasodium Glutamate Diacetate, Rosmarinus Officinalis Extract</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1 flagged ingredient(s) incl. Titanium Dioxide. Escalation: PFAS, heavy metals.</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr"/>
+          <t>1 flagged ingredient(s) in the printed list (Sodium Cocoyl Isethionate); tier applies to the printed subset only. 5 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 5 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1038,26 +1078,34 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Puberty Safe</t>
+          <t>Use Caution</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Sodium Cocoyl Isethionate [1]</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Sodium Cocoamphoacetate, Hydrolyzed Jojoba Esters</t>
+          <t>unknown — manual review needed: Sodium Cocoamphoacetate, Tetrasodium Glutamate Diacetate, Hydrolyzed Jojoba Esters, Aloe Barbadensis Leaf Juice, Arctium Lappa Root Extract, Chamomilla Recutita Flower Extract</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
-          <t>No flagged ingredients present per reference.</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr"/>
+          <t>1 flagged ingredient(s) in the printed list (Sodium Cocoyl Isethionate); tier applies to the printed subset only. 6 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 6 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1100,22 +1148,26 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Cocamidopropyl Hydroxysultaine [1,4] / Parfum [1,2,4,8]</t>
+          <t>Cocamidopropyl Hydroxysultaine [1,4] / Parfum [1,2,4,8] (fragrance without disclosure)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Sodium Methyl 2-Sulfolaurate, Cyamopsis Tetragonoloba Gum, Disodium 2-Sulfolaurate, Hydrolyzed Jojoba Esters</t>
+          <t>unknown — manual review needed: Sodium Lauroyl Sarcosinate, Sodium Methyl 2-Sulfolaurate, Cyamopsis Tetragonoloba Gum, Disodium 2-Sulfolaurate, Tetrasodium Glutamate Diacetate, Hydrolyzed Jojoba Esters, Aloe Barbadensis Leaf Juice, Butyrospermum Parkii Butter, Arctium Lappa Root Extract, Chamomilla Recutita Flower Extract</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2 flagged ingredient(s) incl. Cocamidopropyl Hydroxysultaine, Parfum.</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr"/>
+          <t>2 flagged ingredient(s) in the printed list (Cocamidopropyl Hydroxysultaine, Parfum); tier applies to the printed subset only. 10 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Identical printed text on 1 other product(s): 365 Liquid Hand Soap Anjou Pear. D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 10 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N12" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1158,22 +1210,26 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Cocamidopropyl Hydroxysultaine [1,4] / Parfum [1,2,4,8]</t>
+          <t>Cocamidopropyl Hydroxysultaine [1,4] / Parfum [1,2,4,8] (fragrance without disclosure)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Sodium Methyl 2-Sulfolaurate, Cyamopsis Tetragonoloba Gum, Disodium 2-Sulfolaurate, Hydrolyzed Jojoba Esters</t>
+          <t>unknown — manual review needed: Sodium Lauroyl Sarcosinate, Sodium Methyl 2-Sulfolaurate, Cyamopsis Tetragonoloba Gum, Disodium 2-Sulfolaurate, Tetrasodium Glutamate Diacetate, Hydrolyzed Jojoba Esters, Aloe Barbadensis Leaf Juice, Butyrospermum Parkii Butter, Arctium Lappa Root Extract, Chamomilla Recutita Flower Extract</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2 flagged ingredient(s) incl. Cocamidopropyl Hydroxysultaine, Parfum.</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr"/>
+          <t>2 flagged ingredient(s) in the printed list (Cocamidopropyl Hydroxysultaine, Parfum); tier applies to the printed subset only. 10 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Identical printed text on 1 other product(s): 365 Liquid Hand Soap. D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 10 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1222,16 +1278,20 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Sodium Methyl 2-Sulfolaurate, Cyamopsis Tetragonoloba Gum, Disodium 2-Sulfolaurate, Hydrolyzed Jojoba Esters</t>
+          <t>unknown — manual review needed: Sodium Lauroyl Sarcosinate, Sodium Methyl 2-Sulfolaurate, Cyamopsis Tetragonoloba Gum, Disodium 2-Sulfolaurate, Tetrasodium Glutamate Diacetate, Hydrolyzed Jojoba Esters, Aloe Barbadensis Leaf Juice, Butyrospermum Parkii Butter, Arctium Lappa Root Extract, Chamomilla Recutita Flower Extract</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1 flagged ingredient(s) incl. Cocamidopropyl Hydroxysultaine.</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr"/>
+          <t>1 flagged ingredient(s) in the printed list (Cocamidopropyl Hydroxysultaine); tier applies to the printed subset only. 10 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 10 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1270,15 +1330,19 @@
         </is>
       </c>
       <c r="G15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Dimethicone [2,6] / Ethylhexylglycerin [4,5] / Parfum [1,2,4,8] / Phenoxyethanol [1,2,4,5,8]</t>
+          <t>Polysorbate 20 [1,2,4,5] / Dimethicone [2,6] / Ethylhexylglycerin [4,5] / Parfum [1,2,4,8] (fragrance without disclosure) / Phenoxyethanol [1,2,4,5,8]</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>unknown — manual review needed: Isopropyl Palmitate, Butyrospermum Parkii Butter, Cocos Nucifera Oil, Cannabis Sativa Seed Oil, Argania Spinosa Kernel Oil, Aloe Barbadensis Leaf Extract, Camellia Sinensis Leaf Extract, Chamomilla Recutita Flower Extract, Cucumis Sativus Fruit Extract, Lavandula Angustifolia Flower Extract, Tocopheryl Acetate, Lecithin, Echinacea Angustifolia Root Extract</t>
+        </is>
+      </c>
       <c r="K15" t="inlineStr">
         <is>
           <t>PFAS, carcinogen in leave-on</t>
@@ -1286,10 +1350,14 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>4 flagged ingredient(s) incl. Dimethicone, Ethylhexylglycerin, Parfum. Escalation: PFAS, carcinogen in leave-on.</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr"/>
+          <t>5 flagged ingredient(s) in the printed list (Polysorbate 20, Dimethicone, Ethylhexylglycerin); tier applies to the printed subset only. 13 unknown ingredient(s) not in reference, excluded from grade. Escalation: PFAS, carcinogen in leave-on.</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Identical printed text on 1 other product(s): 365 Maximum Moisture Lotion Lavender. D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 13 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1328,15 +1396,19 @@
         </is>
       </c>
       <c r="G16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Dimethicone [2,6] / Ethylhexylglycerin [4,5] / Parfum [1,2,4,8] / Phenoxyethanol [1,2,4,5,8]</t>
+          <t>Polysorbate 20 [1,2,4,5] / Dimethicone [2,6] / Ethylhexylglycerin [4,5] / Parfum [1,2,4,8] (fragrance without disclosure) / Phenoxyethanol [1,2,4,5,8]</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>unknown — manual review needed: Isopropyl Palmitate, Butyrospermum Parkii Butter, Cocos Nucifera Oil, Cannabis Sativa Seed Oil, Argania Spinosa Kernel Oil, Aloe Barbadensis Leaf Extract, Camellia Sinensis Leaf Extract, Chamomilla Recutita Flower Extract, Cucumis Sativus Fruit Extract, Lavandula Angustifolia Flower Extract, Tocopheryl Acetate, Lecithin, Echinacea Angustifolia Root Extract</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
           <t>PFAS, carcinogen in leave-on</t>
@@ -1344,10 +1416,14 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>4 flagged ingredient(s) incl. Dimethicone, Ethylhexylglycerin, Parfum. Escalation: PFAS, carcinogen in leave-on.</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
+          <t>5 flagged ingredient(s) in the printed list (Polysorbate 20, Dimethicone, Ethylhexylglycerin); tier applies to the printed subset only. 13 unknown ingredient(s) not in reference, excluded from grade. Escalation: PFAS, carcinogen in leave-on.</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Identical printed text on 1 other product(s): 365 Maximum Moisture Lotion. D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 13 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N16" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1386,17 +1462,17 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Dimethicone [2,6] / Phenoxyethanol [1,2,4,5,8]</t>
+          <t>Propanediol [4] / Dimethicone [2,6] / Phenoxyethanol [1,2,4,5,8]</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Sorbitan Caprylate, Sodium Stearoyl Glutamate</t>
+          <t>unknown — manual review needed: Caprylic/Capric Triglyceride, Isopropyl Palmitate, Butyrospermum Parkii Butter, Sorbitan Caprylate, Colloidal Oatmeal, Acrylates/C10-30 Alkyl Acrylate Crosspolymer, Sodium Stearoyl Glutamate, Sodium Hydroxide, Avena Sativa Kernel Extract, Aloe Barbadensis Leaf Juice</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -1406,10 +1482,14 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2 flagged ingredient(s) incl. Dimethicone, Phenoxyethanol. Escalation: PFAS, carcinogen in leave-on.</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr"/>
+          <t>3 flagged ingredient(s) in the printed list (Propanediol, Dimethicone, Phenoxyethanol); tier applies to the printed subset only. 10 unknown ingredient(s) not in reference, excluded from grade. Escalation: PFAS, carcinogen in leave-on.</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 10 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1448,15 +1528,19 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Phenoxyethanol [1,2,4,5,8] / Dimethicone [2,6] / Ethylhexylglycerin [4,5]</t>
+          <t>Polysorbate 60 [1,2,4,5] / Phenoxyethanol [1,2,4,5,8] / Dimethicone [2,6] / Ethylhexylglycerin [4,5]</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>unknown — manual review needed: Isopropyl Palmitate, Caprylic/Capric Triglyceride, Sodium Hydroxide, Butyrospermum Parkii Butter, Lavandula Angustifolia Flower Extract, Calendula Officinalis Flower Extract, Helianthus Annuus Seed Oil, Spiraea Ulmaria Leaf Extract</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>PFAS, carcinogen in leave-on</t>
@@ -1464,10 +1548,14 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>3 flagged ingredient(s) incl. Phenoxyethanol, Dimethicone, Ethylhexylglycerin. Escalation: PFAS, carcinogen in leave-on.</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr"/>
+          <t>4 flagged ingredient(s) in the printed list (Polysorbate 60, Phenoxyethanol, Dimethicone); tier applies to the printed subset only. 8 unknown ingredient(s) not in reference, excluded from grade. Escalation: PFAS, carcinogen in leave-on.</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 8 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1502,7 +1590,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Puberty Safe</t>
+          <t>Use Caution</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1512,16 +1600,20 @@
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Zinc Oxide</t>
+          <t>unknown — manual review needed: Helianthus Annuus Seed Oil, Simmondsia Chinensis Seed Oil, Cocos Nucifera Oil</t>
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
-          <t>No flagged ingredients present per reference.</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
+          <t>No flagged ingredients in the printed list per reference and rubric conditionals. 3 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>3 unknown ingredient(s) excluded from flags (2026-10-17). Puberty Safe requires zero unknown ingredients: 3 unknown ingredient(s) move this product to Use Caution (2026-10-17 practitioner rule). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N19" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1570,16 +1662,20 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Sodium Methyl 2-Sulfolaurate, Cocoyl Methyl Glucamide, Cetyl Betaine, Capryloyl/Caproyl Anhydro Methyl Glucamide, Disodium 2-Sulfolaurate</t>
+          <t>unknown — manual review needed: Sodium Methyl 2-Sulfolaurate, Cocoyl Methyl Glucamide, Cetyl Betaine, Capryloyl/Caproyl Anhydro Methyl Glucamide, Disodium 2-Sulfolaurate, Tetrasodium Glutamate Diacetate, Aloe Barbadensis Leaf Juice</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
-          <t>1 flagged ingredient(s) incl. Cocamidopropyl Hydroxysultaine.</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr"/>
+          <t>1 flagged ingredient(s) in the printed list (Cocamidopropyl Hydroxysultaine); tier applies to the printed subset only. 7 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 7 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1618,26 +1714,30 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Butylene Glycol [1,2] / Parfum [1,2,4,8] / Phenoxyethanol [1,2,4,5,8] / Ethylhexylglycerin [4,5]</t>
+          <t>Butylene Glycol [1,2] / Parfum [1,2,4,8] (fragrance without disclosure) / Phenoxyethanol [1,2,4,5,8] / Potassium Hydroxide [4] / Carbomer [1,4,6] / Ethylhexylglycerin [4,5]</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Juglans Regia Shell Powder, Sorbitan Sesquioleate</t>
+          <t>unknown — manual review needed: Stearic Acid, Juglans Regia Shell Powder, Caprylic/Capric Triglyceride, Carthamus Tinctorius Seed Oil, Coco-Betaine, Butyrospermum Parkii Butter, Olea Europaea Fruit Oil, Sorbitan Sesquioleate, Hydrogenated Lecithin, Cocos Nucifera Oil, Glyceryl Stearate, Acrylates/C10-30 Alkyl Acrylate Crosspolymer, Behenic Acid, Myristic Acid, Prunus Armeniaca Fruit Extract</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
-          <t>4 flagged ingredient(s) incl. Butylene Glycol, Parfum, Phenoxyethanol.</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
+          <t>6 flagged ingredient(s) in the printed list (Butylene Glycol, Parfum, Phenoxyethanol); tier applies to the printed subset only. 15 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 15 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N21" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1676,15 +1776,19 @@
         </is>
       </c>
       <c r="G22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Phenethyl Alcohol [4,5,8] / Phenoxyethanol [1,2,4,5,8]</t>
+          <t>Pelargonium Graveolens Flower Oil [2] (inferred: -nium quat) / Phenethyl Alcohol [4,5,8] / Phenoxyethanol [1,2,4,5,8]</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>unknown — manual review needed: Hamamelis Virginiana Water, Aloe Barbadensis Leaf Juice, Rosa Damascena Flower Water, Rose Flower Oil, Camellia Sinensis Leaf Extract, Eugenia Caryophyllus Leaf Oil, Anhydroxylitol, Xylitylglucoside, Xylitol, Gluconolactone</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
           <t>carcinogen in leave-on</t>
@@ -1692,10 +1796,14 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2 flagged ingredient(s) incl. Phenethyl Alcohol, Phenoxyethanol. Escalation: carcinogen in leave-on.</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
+          <t>3 flagged ingredient(s) in the printed list (Pelargonium Graveolens Flower Oil, Phenethyl Alcohol, Phenoxyethanol); tier applies to the printed subset only. 10 unknown ingredient(s) not in reference, excluded from grade. Escalation: carcinogen in leave-on.</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 10 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N22" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1734,17 +1842,17 @@
         </is>
       </c>
       <c r="G23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Alcohol [inferred: alcohol] [4] / Phenoxyethanol [1,2,4,5,8]</t>
+          <t>Alcohol [4] (inferred: alcohol) / Polysorbate 20 [1,2,4,5] / Phenoxyethanol [1,2,4,5,8]</t>
         </is>
       </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Caprylic/Capric Glycerides Polyglyceryl-10 Esters, Hydrolyzed Algin, Ethyl Lauroyl Arginate Hcl, Sarcosine</t>
+          <t>unknown — manual review needed: Aloe Barbadensis Leaf Juice, Xylitylglucoside, Xylitol, Caprylic/Capric Glycerides Polyglyceryl-10 Esters, Hamamelis Virginiana Water, Camellia Sinensis Leaf Extract, Capryloyl Glycine, Hydrolyzed Algin, Ethyl Lauroyl Arginate Hcl, Citrus Paradisi Fruit Extract, Cucumis Melo Fruit Extract, Citrus Aurantium Dulcis Peel Extract, Theobroma Cacao Extract, Citrus Tangerina Peel Extract, Cinnamomum Zeylanicum Bark Extract, Chlorella Vulgaris Extract, Sarcosine, Sea Water, Anhydroxylitol, Gluconolactone</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -1754,10 +1862,14 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2 flagged ingredient(s) incl. Alcohol, Phenoxyethanol. Escalation: carcinogen in leave-on.</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr"/>
+          <t>3 flagged ingredient(s) in the printed list (Alcohol, Polysorbate 20, Phenoxyethanol); tier applies to the printed subset only. 20 unknown ingredient(s) not in reference, excluded from grade. Escalation: carcinogen in leave-on.</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 20 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N23" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1792,7 +1904,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Puberty Safe</t>
+          <t>Use Caution</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1802,16 +1914,20 @@
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Aroma, Honey</t>
+          <t>unknown — manual review needed: Cocos Nucifera Oil, Olea Europaea Fruit Oil, Butyrospermum Parkii Butter, Aroma, Theobroma Cacao Seed Butter, Cannabis Sativa Seed Oil, Honey</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
-          <t>No flagged ingredients present per reference.</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
+          <t>No flagged ingredients in the printed list per reference and rubric conditionals. 7 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>7 unknown ingredient(s) excluded from flags (2026-10-17). Puberty Safe requires zero unknown ingredients: 7 unknown ingredient(s) move this product to Use Caution (2026-10-17 practitioner rule). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N24" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1846,7 +1962,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Puberty Safe</t>
+          <t>Use Caution</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -1854,14 +1970,22 @@
       </c>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>unknown — manual review needed: Prunus Amygdalus Dulcis Oil</t>
+        </is>
+      </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
-          <t>No flagged ingredients present per reference.</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
+          <t>No flagged ingredients in the printed list per reference and rubric conditionals. 1 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>1 unknown ingredient(s) excluded from flags (2026-10-17). Puberty Safe requires zero unknown ingredients: 1 unknown ingredient(s) move this product to Use Caution (2026-10-17 practitioner rule). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N25" t="inlineStr">
         <is>
           <t>complete</t>
@@ -1896,7 +2020,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Puberty Safe</t>
+          <t>Use Caution</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -1906,16 +2030,20 @@
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Sodium Monofluorophosphate 0.76% , Calcium Carbonate, Hydrated Silica, Natural Flavor</t>
+          <t>unknown — manual review needed: Sodium Monofluorophosphate, Calcium Carbonate, Hydrated Silica, Xylitol, Carrageenan, Cannabis Sativa (Hemp) Seed Oil, Sodium Lauroyl Sarcosinate, Natural Flavor, Zinc Citrate</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
-          <t>No flagged ingredients present per reference.</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr"/>
+          <t>No flagged ingredients in the printed list per reference and rubric conditionals. 9 unknown ingredient(s) not in reference, excluded from grade.</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>D6: glycerin is a caution ingredient (not a flag); it floors a Puberty Safe product at Use Caution. 9 unknown ingredient(s) excluded from flags (2026-10-17). Ingredient source: Carried over from prior wf365 audit (xlsx); verbatim text not re-scraped 2026-10-17.</t>
+        </is>
+      </c>
       <c r="N26" t="inlineStr">
         <is>
           <t>complete</t>

</xml_diff>